<commit_message>
Simplificación de lógica de validación de trámites.
Se actualiza `procesar_tramites.py` para:
- Validar status 200 de URLs.
- Verificar presencia de "Consulta en línea".
- Remover extracción de metadatos adicionales (Tipo, Nombre, Área).
- Mantener reporte Excel simplificado.

Co-authored-by: JohanLieberth <212394673+JohanLieberth@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resultado_tramites.xlsx
+++ b/resultado_tramites.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,21 +429,6 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Área Responsable</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
           <t>Tiene Consulta en Línea</t>
         </is>
       </c>
@@ -461,21 +446,6 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -493,21 +463,6 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -525,21 +480,6 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -557,21 +497,6 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -589,21 +514,6 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -621,21 +531,6 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -653,21 +548,6 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -685,21 +565,6 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -717,21 +582,6 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -748,21 +598,6 @@
         </is>
       </c>
       <c r="C11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Actualización de lógica para conteo de 'Consulta en línea'.
Se modifica `procesar_tramites.py` para:
- Centrarse exclusivamente en la detección de 'Consulta en línea'.
- Mostrar el total acumulado de URLs que cuentan con esta información y las que no.
- Generar el reporte Excel con el estado final de cada URL.

Co-authored-by: JohanLieberth <212394673+JohanLieberth@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resultado_tramites.xlsx
+++ b/resultado_tramites.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,11 +424,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>Tiene Consulta en Línea</t>
         </is>
       </c>
@@ -441,11 +436,6 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -458,11 +448,6 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -475,11 +460,6 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -492,11 +472,6 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -509,11 +484,6 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -526,11 +496,6 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -543,11 +508,6 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -560,11 +520,6 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -577,11 +532,6 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
@@ -593,11 +543,6 @@
         </is>
       </c>
       <c r="B11" t="inlineStr">
-        <is>
-          <t>Bloqueado (Captcha)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Mejora de detección y soporte para entrada Excel en el scraper de Mérida.
Se actualiza `procesar_tramites.py` para:
- Leer lista de URLs desde `urls_entrada.xlsx`.
- Mejorar la lógica de detección de 'Consulta en línea' incluyendo variantes como 'Trámite en línea'.
- Reportar explícitamente bloqueos por Captcha.
- Mostrar resumen de totales (con/sin dato y bloqueados).

Co-authored-by: JohanLieberth <212394673+JohanLieberth@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resultado_tramites.xlsx
+++ b/resultado_tramites.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,6 +424,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Tiene Consulta en Línea</t>
         </is>
       </c>
@@ -436,6 +441,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Bloqueado (Captcha)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
@@ -448,101 +458,10 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/568</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/781</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/325</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/534</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/508</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/565</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/327</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>https://isla.merida.gob.mx/serviciosinternet/tramites/detalle/458</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+          <t>Bloqueado (Captcha)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>